<commit_message>
Main project files added
</commit_message>
<xml_diff>
--- a/GroceryApplicationProject/src/test/resources/Testdata.xlsx
+++ b/GroceryApplicationProject/src/test/resources/Testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\git\GroceryApplicationProject\GroceryApplicationProject\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33FF8857-15BC-4E93-BE4E-DDF8B5075237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378687E8-15CD-4319-B335-D61140B5A65F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPage" sheetId="1" r:id="rId1"/>
@@ -107,10 +107,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -438,13 +439,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E64FE51-9C63-432F-B590-2C7FD2CB0E35}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -454,8 +455,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D1" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -463,7 +467,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -471,7 +475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>

</xml_diff>